<commit_message>
Refactoed- Now the User profile are added and the authendication is created
</commit_message>
<xml_diff>
--- a/backend/profile_data.xlsx
+++ b/backend/profile_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
   <si>
     <t>Role</t>
   </si>
@@ -116,6 +116,90 @@
   </si>
   <si>
     <t>2026-08-12T17:18:33Z</t>
+  </si>
+  <si>
+    <t>2026-08-12T23:10:14Z</t>
+  </si>
+  <si>
+    <t>PROF-002</t>
+  </si>
+  <si>
+    <t>Mukesh T</t>
+  </si>
+  <si>
+    <t>Principal DBA / MLOps</t>
+  </si>
+  <si>
+    <t>mtdev8386@gmail.com</t>
+  </si>
+  <si>
+    <t>Backend /Systems</t>
+  </si>
+  <si>
+    <t>https://media.licdn.com/dms/image/v2/D5603AQE4KLkWLfRCVw/profile-displayphoto-scale_400_400/B56ZjwuZI2HMAo-/0/1756385352773?e=1788393600&amp;v=beta&amp;t=DtexI3bPy8_EZTPd8k9Eq6fVAvWV5NDBBxa0EGuQ7JQ</t>
+  </si>
+  <si>
+    <t>#10B981</t>
+  </si>
+  <si>
+    <t>a5266239ab5a99c8456d926461b67c9953887f857fd3a7d86dc399e5012b9a5d</t>
+  </si>
+  <si>
+    <t>2026-08-13T00:02:15Z</t>
+  </si>
+  <si>
+    <t>PROF-003</t>
+  </si>
+  <si>
+    <t>Prithiv Krishna G</t>
+  </si>
+  <si>
+    <t>Forward Deployment Engineer</t>
+  </si>
+  <si>
+    <t>prithivkrishna1116@gmail.com</t>
+  </si>
+  <si>
+    <t>CIC / Deployment</t>
+  </si>
+  <si>
+    <t>https://media.licdn.com/dms/image/v2/D5603AQGI7IvLhdydYw/profile-displayphoto-scale_400_400/B56ZzJ1xcxH8Ag-/0/1772912845281?e=1788393600&amp;v=beta&amp;t=5Dv6ZFeIxF8k3NTQ7QlcF3aIyxcc8W9F4dcC9_Lkme0</t>
+  </si>
+  <si>
+    <t>#3B82F6</t>
+  </si>
+  <si>
+    <t>aeb32cfe00d196040e9758c276853282721fbd222038a54e9ae04d6686066e1b</t>
+  </si>
+  <si>
+    <t>2026-08-13T00:05:18Z</t>
+  </si>
+  <si>
+    <t>PROF-004</t>
+  </si>
+  <si>
+    <t>MOHAMED SUHAIL J</t>
+  </si>
+  <si>
+    <t>Business analyst</t>
+  </si>
+  <si>
+    <t>mohamedsuhails507@gmail.com</t>
+  </si>
+  <si>
+    <t>Gen AI</t>
+  </si>
+  <si>
+    <t>https://media.licdn.com/dms/image/v2/D5603AQFzHYv-WMLFNQ/profile-displayphoto-shrink_400_400/B56ZU7f8K7GUAs-/0/1740459984578?e=1788393600&amp;v=beta&amp;t=BX0iwSCbFRUTTQdBnNUXk2gfl5SK5-lwUoyIsX4BxKk</t>
+  </si>
+  <si>
+    <t>#F59E0B</t>
+  </si>
+  <si>
+    <t>594686bcfe8a1c52aa5c6ab2feadeac31c7fbc9815ad68487b60d946a12e4765</t>
+  </si>
+  <si>
+    <t>2026-08-13T00:07:06Z</t>
   </si>
 </sst>
 </file>
@@ -492,7 +576,94 @@
         <v>31</v>
       </c>
       <c r="I2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G3" t="s">
+        <v>41</v>
+      </c>
+      <c r="H3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" t="s">
+        <v>57</v>
+      </c>
+      <c r="F5" t="s">
+        <v>58</v>
+      </c>
+      <c r="G5" t="s">
+        <v>59</v>
+      </c>
+      <c r="H5" t="s">
+        <v>60</v>
+      </c>
+      <c r="I5" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>